<commit_message>
GOODLUCK DEFENSE ft cert adjust 2
</commit_message>
<xml_diff>
--- a/myapp/cert_templates/Completion_Certificate.xlsx
+++ b/myapp/cert_templates/Completion_Certificate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\thesis_osa\myapp\cert_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9130862-E840-49A0-8722-95182F41EBA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B63B18-63F0-4BA0-8539-069130CE6384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -100,12 +100,6 @@
     <t>TECHNOLOGICAL UNIVERSITY OF THE PHILIPPINES</t>
   </si>
   <si>
-    <t xml:space="preserve">                   CAVITE CAMPUS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">                 CQT. Ave., Salawag City of Dasmariñas City, Cavite</t>
-  </si>
-  <si>
     <t>CERTIFICATION OF COMMUNITY SERVICE COMPLETED</t>
   </si>
   <si>
@@ -128,6 +122,12 @@
   </si>
   <si>
     <t>Head, Office of Student Affairs</t>
+  </si>
+  <si>
+    <t>CAVITE CAMPUS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  CQT. Ave., Salawag City of Dasmariñas City, Cavite</t>
   </si>
 </sst>
 </file>
@@ -202,31 +202,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -235,15 +220,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -252,6 +228,27 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -274,16 +271,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>97200</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>63360</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>109106</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>39547</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>532800</xdr:colOff>
+      <xdr:colOff>270862</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>107280</xdr:rowOff>
+      <xdr:rowOff>148951</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -302,8 +299,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="177840" y="63360"/>
-          <a:ext cx="435600" cy="434520"/>
+          <a:off x="109106" y="105031"/>
+          <a:ext cx="435600" cy="430873"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -503,74 +500,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="5">
         <v>45699</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="4" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="4" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="6">
         <v>20</v>
       </c>
     </row>
@@ -585,7 +582,7 @@
   <dimension ref="A1:E21"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="12.75" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="1.140625" customWidth="1"/>
+    <col min="1" max="1" width="4.140625" customWidth="1"/>
     <col min="2" max="2" width="27.28515625" customWidth="1"/>
     <col min="3" max="3" width="3.5703125" customWidth="1"/>
     <col min="4" max="4" width="20.28515625" customWidth="1"/>
@@ -595,144 +592,144 @@
   <sheetData>
     <row r="1" spans="2:4" ht="5.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B3" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
+      <c r="B3" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
     </row>
     <row r="4" spans="2:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
+      <c r="B4" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.2"/>
     <row r="6" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B6" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
+      <c r="B6" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="13" t="str">
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="1" t="str">
         <f>TEXT(date,"mmmm d, yyyy")</f>
         <v>February 11, 2025</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.2"/>
     <row r="10" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B10" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
+      <c r="B10" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B11" s="15" t="str">
+      <c r="B11" s="7" t="str">
         <f>student_name</f>
         <v>Lord Jaisson Riberal</v>
       </c>
-      <c r="C11" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="D11" s="16" t="str">
+      <c r="C11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="8" t="str">
         <f>program</f>
         <v>BET-COET</v>
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+    </row>
+    <row r="13" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B13" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+    </row>
+    <row r="14" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B14" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-    </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B13" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-    </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B14" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="C14" s="13">
+      <c r="C14" s="1">
         <f>hours</f>
         <v>20</v>
       </c>
-      <c r="D14" s="9" t="s">
-        <v>25</v>
+      <c r="D14" s="4" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B15" s="3" t="str">
+      <c r="B15" s="12" t="str">
         <f>"community service from " &amp; TEXT(start_date,"mmmm d, yyyy") &amp;
 " to " &amp; TEXT(end_date,"mmmm d, yyyy") &amp;
 " and is hereby cleared in this office of such violation."</f>
         <v>community service from November 10. 2025 to November 20, 2025 and is hereby cleared in this office of such violation.</v>
       </c>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.2"/>
     <row r="19" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B19" s="1" t="str">
+      <c r="B19" s="13" t="str">
         <f>osa_head</f>
         <v>Beverly M. de Vega</v>
       </c>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B20" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
+      <c r="B20" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B10:D10"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="B15:D16"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B10:D10"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.98402777777777795" right="0.98402777777777795" top="0.31527777777777799" bottom="0.98402777777777795" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
GOODLUCK DEFENSE ft cert adjust 3
</commit_message>
<xml_diff>
--- a/myapp/cert_templates/Completion_Certificate.xlsx
+++ b/myapp/cert_templates/Completion_Certificate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\thesis_osa\myapp\cert_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B63B18-63F0-4BA0-8539-069130CE6384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE4D8886-1622-453F-A60D-279E387FA74E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -229,25 +229,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -271,16 +271,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>109106</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>39547</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>73387</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>51453</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>270862</xdr:colOff>
+      <xdr:colOff>508987</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>148951</xdr:rowOff>
+      <xdr:rowOff>95373</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -299,7 +299,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="109106" y="105031"/>
+          <a:off x="347231" y="51453"/>
           <a:ext cx="435600" cy="430873"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -585,40 +585,40 @@
     <col min="1" max="1" width="4.140625" customWidth="1"/>
     <col min="2" max="2" width="27.28515625" customWidth="1"/>
     <col min="3" max="3" width="3.5703125" customWidth="1"/>
-    <col min="4" max="4" width="20.28515625" customWidth="1"/>
+    <col min="4" max="4" width="28.5703125" customWidth="1"/>
     <col min="5" max="5" width="3.140625" customWidth="1"/>
     <col min="6" max="16384" width="9.140625" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:4" ht="5.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
     </row>
     <row r="4" spans="2:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.2"/>
     <row r="6" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="16"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B7" s="3"/>
@@ -635,11 +635,11 @@
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.2"/>
     <row r="10" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B11" s="7" t="str">
@@ -655,18 +655,18 @@
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B14" s="9" t="s">
@@ -681,55 +681,55 @@
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B15" s="12" t="str">
+      <c r="B15" s="15" t="str">
         <f>"community service from " &amp; TEXT(start_date,"mmmm d, yyyy") &amp;
 " to " &amp; TEXT(end_date,"mmmm d, yyyy") &amp;
 " and is hereby cleared in this office of such violation."</f>
         <v>community service from November 10. 2025 to November 20, 2025 and is hereby cleared in this office of such violation.</v>
       </c>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.2"/>
     <row r="19" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B19" s="13" t="str">
+      <c r="B19" s="16" t="str">
         <f>osa_head</f>
         <v>Beverly M. de Vega</v>
       </c>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B10:D10"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="B15:D16"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B10:D10"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.98402777777777795" right="0.98402777777777795" top="0.31527777777777799" bottom="0.98402777777777795" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>